<commit_message>
Auto update Pengadaan 2026-09-11 08:08:21
</commit_message>
<xml_diff>
--- a/output/tepra/2026/Tepra Kobar_Progres PBJ tahun 2026 (2026-09-11).xlsx
+++ b/output/tepra/2026/Tepra Kobar_Progres PBJ tahun 2026 (2026-09-11).xlsx
@@ -3345,22 +3345,22 @@
         <v>1352438071</v>
       </c>
       <c r="E76" s="7" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F76" s="9" t="n">
-        <v>183633343</v>
+        <v>189483343</v>
       </c>
       <c r="G76" s="7" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="H76" s="9" t="n">
-        <v>160778238</v>
+        <v>162128238</v>
       </c>
       <c r="I76" s="7" t="n">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="J76" s="9" t="n">
-        <v>1168804728</v>
+        <v>1162954728</v>
       </c>
     </row>
     <row r="77" ht="45" customHeight="1">
@@ -3377,22 +3377,22 @@
         <v>32602025242</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="F77" s="13" t="n">
-        <v>6227658417</v>
+        <v>6233508417</v>
       </c>
       <c r="G77" s="12" t="n">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>5746517118.6</v>
+        <v>5747867118.6</v>
       </c>
       <c r="I77" s="12" t="n">
-        <v>3548</v>
+        <v>3547</v>
       </c>
       <c r="J77" s="13" t="n">
-        <v>26374366825</v>
+        <v>26368516825</v>
       </c>
     </row>
   </sheetData>
@@ -4844,10 +4844,10 @@
         <v>14949019060.4</v>
       </c>
       <c r="I29" s="4" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="J29" s="11" t="n">
-        <v>10381028359</v>
+        <v>10437022087</v>
       </c>
       <c r="K29" s="4" t="n">
         <v>1</v>
@@ -7578,10 +7578,10 @@
         <v>61604703796.41</v>
       </c>
       <c r="I77" s="12" t="n">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="J77" s="13" t="n">
-        <v>29094027075</v>
+        <v>29150020803</v>
       </c>
       <c r="K77" s="12" t="n">
         <v>10</v>
@@ -8395,19 +8395,19 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D17" s="11" t="n">
-        <v>26120170739</v>
+        <v>26485477939</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F17" s="11" t="n">
-        <v>26120170739</v>
+        <v>26485477939</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H17" s="11" t="n">
         <v>26035273641</v>
@@ -9059,10 +9059,10 @@
         </is>
       </c>
       <c r="C29" s="4" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D29" s="11" t="n">
-        <v>11886677646</v>
+        <v>11521370446</v>
       </c>
       <c r="E29" s="4" t="n">
         <v>22</v>
@@ -9093,10 +9093,10 @@
         </is>
       </c>
       <c r="M29" s="4" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="N29" s="11" t="n">
-        <v>4343051552</v>
+        <v>3977744352</v>
       </c>
     </row>
     <row r="30" ht="45" customHeight="1">
@@ -12047,13 +12047,13 @@
         <v>179959416808</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F77" s="13" t="n">
-        <v>140927873778</v>
+        <v>141293180978</v>
       </c>
       <c r="G77" s="12" t="n">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="H77" s="13" t="n">
         <v>69572168800.98001</v>
@@ -12071,10 +12071,10 @@
         <v>3046617077</v>
       </c>
       <c r="M77" s="12" t="n">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="N77" s="13" t="n">
-        <v>39031543030</v>
+        <v>38666235830</v>
       </c>
     </row>
   </sheetData>

</xml_diff>